<commit_message>
Refactor yearly data handling and update figures
Moved yearly data processing to a dedicated section, added consistency checks and filling for missing yearly data based on monthly data. Updated normalization logic, plot breaks, and output tables. Regenerated figure and appendix files to reflect these changes.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig1.xlsx
+++ b/Outcome/Publish/figure_data/fig1.xlsx
@@ -30502,7 +30502,7 @@
         <v>59</v>
       </c>
       <c r="C44" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -30829,7 +30829,7 @@
         <v>1.54747733185568</v>
       </c>
       <c r="D24" t="n">
-        <v>1.20316782688397</v>
+        <v>1.18225686080645</v>
       </c>
     </row>
     <row r="25">
@@ -30843,7 +30843,7 @@
         <v>0.769759973291176</v>
       </c>
       <c r="D25" t="n">
-        <v>0.00852283888286707</v>
+        <v>0.0153517048076012</v>
       </c>
     </row>
     <row r="26">
@@ -30857,7 +30857,7 @@
         <v>0.764211580412933</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>0.00702676749479686</v>
       </c>
     </row>
     <row r="27">
@@ -30867,8 +30867,12 @@
       <c r="B27" t="n">
         <v>2016</v>
       </c>
-      <c r="C27"/>
-      <c r="D27"/>
+      <c r="C27" t="n">
+        <v>0.759528389986353</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -30881,7 +30885,7 @@
         <v>1.36239726332537</v>
       </c>
       <c r="D28" t="n">
-        <v>0.918867915336739</v>
+        <v>0.904558434942233</v>
       </c>
     </row>
     <row r="29">
@@ -30895,7 +30899,7 @@
         <v>2.47195547204809</v>
       </c>
       <c r="D29" t="n">
-        <v>2.62325079730394</v>
+        <v>2.56936529617678</v>
       </c>
     </row>
     <row r="30">
@@ -30909,7 +30913,7 @@
         <v>2.31221004596997</v>
       </c>
       <c r="D30" t="n">
-        <v>2.37786721351384</v>
+        <v>2.32967955522603</v>
       </c>
     </row>
     <row r="31">
@@ -30923,7 +30927,7 @@
         <v>1.65730462815425</v>
       </c>
       <c r="D31" t="n">
-        <v>1.37187259812757</v>
+        <v>1.34704428249493</v>
       </c>
     </row>
     <row r="32">
@@ -30937,7 +30941,7 @@
         <v>1.05773602212046</v>
       </c>
       <c r="D32" t="n">
-        <v>0.450880386402795</v>
+        <v>0.447437645133441</v>
       </c>
     </row>
     <row r="33">
@@ -30951,7 +30955,7 @@
         <v>2.26822666425348</v>
       </c>
       <c r="D33" t="n">
-        <v>2.31030471674774</v>
+        <v>2.26368586955341</v>
       </c>
     </row>
     <row r="34">
@@ -30965,7 +30969,7 @@
         <v>2.31320314050328</v>
       </c>
       <c r="D34" t="n">
-        <v>2.37939269753932</v>
+        <v>2.33116961728849</v>
       </c>
     </row>
     <row r="35">
@@ -30979,7 +30983,7 @@
         <v>1.07949479890153</v>
       </c>
       <c r="D35" t="n">
-        <v>0.484303857462404</v>
+        <v>0.480085018288286</v>
       </c>
     </row>
     <row r="36">
@@ -40994,8 +40998,12 @@
       <c r="B27" t="n">
         <v>2016</v>
       </c>
-      <c r="C27"/>
-      <c r="D27"/>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">

</xml_diff>

<commit_message>
Update figures, data, and analysis results
Refreshed published figures (fig1, fig2, fig3), their associated data files, appendix results, and the month.RData analysis output to reflect latest results and visualizations.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig1.xlsx
+++ b/Outcome/Publish/figure_data/fig1.xlsx
@@ -220,9 +220,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -259,7 +257,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Update appendix data and forecast outputs
Added Best_model_outcome.xlsx and updated multiple appendix and supplementary files, including forecast CSVs and figure data. Removed obsolete forecast files for Encephalitis, HDV, Liver fluke, and Measles. Updated R scripts and RData files to reflect new model results and visualizations.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig1.xlsx
+++ b/Outcome/Publish/figure_data/fig1.xlsx
@@ -220,7 +220,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -257,7 +259,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>